<commit_message>
Clarify NC uncertainty boundary panel
</commit_message>
<xml_diff>
--- a/outputs/source_data/nc_source_data_v1.xlsx
+++ b/outputs/source_data/nc_source_data_v1.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rea14bedda12e4d03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig1_TaskMatrix" sheetId="2" r:id="R04fc19902c5f4984"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2_EarlyWindow" sheetId="3" r:id="Rd42b7d0790584e6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig3_Heldout" sheetId="4" r:id="Rd52ed75e4d7a4fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig3_BootstrapCI" sheetId="5" r:id="Re8f8b2e940d245a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig3_TailAudit" sheetId="6" r:id="R7a47aa9ddfd24fea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig4_ClassicalUnc" sheetId="7" r:id="R66f81ef0f7a34ca6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig4_CalSize" sheetId="8" r:id="R80037d8616a9455e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig5_Residuals" sheetId="9" r:id="R8705216dd5794f38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig6_PhaseAudit" sheetId="10" r:id="Rf21ecd5de3b44d81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig7_Boundary" sheetId="11" r:id="Ra6772d19b53946a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_FeatureGroups" sheetId="12" r:id="Rd9e9a6c289d043ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_ESM_Onset" sheetId="13" r:id="Rd362017b193f4d24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_ESM_Spotcheck" sheetId="14" r:id="Rf99b39229997499f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_EarlyPeak" sheetId="15" r:id="R2c72ad15bf59460e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_PhaseTable" sheetId="16" r:id="R96b7aa85645d4e38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R25fbd3d74bf44ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig1_TaskMatrix" sheetId="2" r:id="Rf2b8b6eb19674109"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2_EarlyWindow" sheetId="3" r:id="R5db33f9e24054be7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig3_Heldout" sheetId="4" r:id="Re49c534f2f194959"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig3_BootstrapCI" sheetId="5" r:id="R0dec80e64cff417f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig3_TailAudit" sheetId="6" r:id="R2246f9ab8c3543be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig4_ClassicalUnc" sheetId="7" r:id="Ra22ff82db5b8455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig4_CalSize" sheetId="8" r:id="R87b9b0e7b3ed4804"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig5_Residuals" sheetId="9" r:id="Rf3e38ccb577a4816"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig6_PhaseAudit" sheetId="10" r:id="R48d33aa1d7084c31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig7_Boundary" sheetId="11" r:id="Ra14bdfb82c9c4582"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_FeatureGroups" sheetId="12" r:id="R770c2e766688420d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_ESM_Onset" sheetId="13" r:id="R126fe0697ddb49cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_ESM_Spotcheck" sheetId="14" r:id="R1afa1fbe8b0146c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_EarlyPeak" sheetId="15" r:id="R5f51a7b536704117"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_PhaseTable" sheetId="16" r:id="Rb9c240d34a0d470b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1474,9 +1474,15 @@
     <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="30" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="34" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="34" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="30" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="30" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="26" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="34" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="30" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="34" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="34" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="34" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -1508,12 +1514,30 @@
         <x:v>zero_shot_conformal_coverage</x:v>
       </x:c>
       <x:c r="J1" s="6" t="str">
+        <x:v>target_domain_interval_width</x:v>
+      </x:c>
+      <x:c r="K1" s="6" t="str">
+        <x:v>target_offset_interval_width</x:v>
+      </x:c>
+      <x:c r="L1" s="6" t="str">
+        <x:v>zero_shot_interval_width</x:v>
+      </x:c>
+      <x:c r="M1" s="6" t="str">
+        <x:v>target_domain_coverage_gap_to_90</x:v>
+      </x:c>
+      <x:c r="N1" s="6" t="str">
+        <x:v>zero_shot_coverage_gap_to_90</x:v>
+      </x:c>
+      <x:c r="O1" s="6" t="str">
+        <x:v>target_offset_coverage_gap_to_90</x:v>
+      </x:c>
+      <x:c r="P1" s="6" t="str">
         <x:v>target_domain_top5_under_factor2_rate</x:v>
       </x:c>
-      <x:c r="K1" s="6" t="str">
+      <x:c r="Q1" s="6" t="str">
         <x:v>target_offset_top5_under_factor2_rate</x:v>
       </x:c>
-      <x:c r="L1" s="6" t="str">
+      <x:c r="R1" s="6" t="str">
         <x:v>zero_shot_top5_under_factor2_rate</x:v>
       </x:c>
     </x:row>
@@ -1542,6 +1566,12 @@
       <x:c r="J2" s="3" t="str"/>
       <x:c r="K2" s="3" t="str"/>
       <x:c r="L2" s="3" t="str"/>
+      <x:c r="M2" s="11" t="str"/>
+      <x:c r="N2" s="11" t="str"/>
+      <x:c r="O2" s="11" t="str"/>
+      <x:c r="P2" s="3" t="str"/>
+      <x:c r="Q2" s="3" t="str"/>
+      <x:c r="R2" s="3" t="str"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="11" t="str">
@@ -1572,12 +1602,30 @@
         <x:v>0.46799999999999997</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
+        <x:v>1.229902297077261</x:v>
+      </x:c>
+      <x:c r="K3" s="3" t="str">
+        <x:v>2.1765535017643094</x:v>
+      </x:c>
+      <x:c r="L3" s="3" t="str">
+        <x:v>1.2277688687743704</x:v>
+      </x:c>
+      <x:c r="M3" s="11" t="str">
+        <x:v>0.004995374653098961</x:v>
+      </x:c>
+      <x:c r="N3" s="11" t="str">
+        <x:v>0.43200000000000005</x:v>
+      </x:c>
+      <x:c r="O3" s="11" t="str">
+        <x:v>-0.0050000000000000044</x:v>
+      </x:c>
+      <x:c r="P3" s="3" t="str">
         <x:v>0.52</x:v>
       </x:c>
-      <x:c r="K3" s="3" t="str">
+      <x:c r="Q3" s="3" t="str">
         <x:v>1.0</x:v>
       </x:c>
-      <x:c r="L3" s="3" t="str">
+      <x:c r="R3" s="3" t="str">
         <x:v>0.5633223684210527</x:v>
       </x:c>
     </x:row>
@@ -1606,6 +1654,12 @@
       <x:c r="J4" s="3" t="str"/>
       <x:c r="K4" s="3" t="str"/>
       <x:c r="L4" s="3" t="str"/>
+      <x:c r="M4" s="11" t="str"/>
+      <x:c r="N4" s="11" t="str"/>
+      <x:c r="O4" s="11" t="str"/>
+      <x:c r="P4" s="3" t="str"/>
+      <x:c r="Q4" s="3" t="str"/>
+      <x:c r="R4" s="3" t="str"/>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="11" t="str">
@@ -1636,12 +1690,30 @@
         <x:v>0.2975498179410791</x:v>
       </x:c>
       <x:c r="J5" s="3" t="str">
+        <x:v>0.8282341110239535</x:v>
+      </x:c>
+      <x:c r="K5" s="3" t="str">
+        <x:v>2.1765535017643094</x:v>
+      </x:c>
+      <x:c r="L5" s="3" t="str">
+        <x:v>0.8261123052615972</x:v>
+      </x:c>
+      <x:c r="M5" s="11" t="str">
+        <x:v>0.0046000000000000485</x:v>
+      </x:c>
+      <x:c r="N5" s="11" t="str">
+        <x:v>0.602450182058921</x:v>
+      </x:c>
+      <x:c r="O5" s="11" t="str">
+        <x:v>-0.0034999999999999476</x:v>
+      </x:c>
+      <x:c r="P5" s="3" t="str">
         <x:v>0.32</x:v>
       </x:c>
-      <x:c r="K5" s="3" t="str">
+      <x:c r="Q5" s="3" t="str">
         <x:v>1.0</x:v>
       </x:c>
-      <x:c r="L5" s="3" t="str">
+      <x:c r="R5" s="3" t="str">
         <x:v>0.44177631578947363</x:v>
       </x:c>
     </x:row>
@@ -1670,6 +1742,12 @@
       <x:c r="J6" s="3" t="str"/>
       <x:c r="K6" s="3" t="str"/>
       <x:c r="L6" s="3" t="str"/>
+      <x:c r="M6" s="11" t="str"/>
+      <x:c r="N6" s="11" t="str"/>
+      <x:c r="O6" s="11" t="str"/>
+      <x:c r="P6" s="3" t="str"/>
+      <x:c r="Q6" s="3" t="str"/>
+      <x:c r="R6" s="3" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>